<commit_message>
Loading the us_states table
</commit_message>
<xml_diff>
--- a/mappings/source_to_bronze/us_zip.xlsx
+++ b/mappings/source_to_bronze/us_zip.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nason\Desktop\Projects\ActiveProjects\BlixHealth\mappings\source_to_bronze\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37AEE5B8-BB71-4F07-8CDE-6629ABC515B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EB860EE-9196-45EC-AE5B-BD36BD2255C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38505" yWindow="0" windowWidth="20130" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="45">
   <si>
     <t>source_database</t>
   </si>
@@ -154,6 +154,12 @@
   </si>
   <si>
     <t>strip</t>
+  </si>
+  <si>
+    <t>current_timestamp</t>
+  </si>
+  <si>
+    <t>no_transform</t>
   </si>
 </sst>
 </file>
@@ -1333,7 +1339,9 @@
         <v>23</v>
       </c>
       <c r="I14" s="7"/>
-      <c r="J14" s="7"/>
+      <c r="J14" s="7" t="s">
+        <v>44</v>
+      </c>
       <c r="K14" s="8"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
@@ -1517,7 +1525,9 @@
         <v>35</v>
       </c>
       <c r="I20" s="7"/>
-      <c r="J20" s="7"/>
+      <c r="J20" s="7" t="s">
+        <v>43</v>
+      </c>
       <c r="K20" s="8"/>
     </row>
   </sheetData>

</xml_diff>